<commit_message>
Checkpoint working Digicon and JMRI tables before Dispatcher auto-run.
Freeze Masters (20260817_015225), tables snapshot, and Pi PanelPro/CATS split so we can roll back without touching live CTC.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/LCOS_Layout_Inventory_v48_signal_ports.xlsx
+++ b/cats/data/LCOS_Layout_Inventory_v48_signal_ports.xlsx
@@ -444,7 +444,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="7.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="12" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -1020,8 +1020,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H259"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:H261"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="15.6640625" bestFit="1" customWidth="1" min="3" max="3"/>
     <col width="17.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>reserved / not Digicon head-mast</t>
+          <t>reserved / not Digicon head-mast | reserved / not Digicon head-mast | reserved / not Digicon head-mast | reserved / not Digicon head-mast</t>
         </is>
       </c>
     </row>
@@ -3843,7 +3843,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>reserved / not Digicon head-mast</t>
+          <t>reserved / not Digicon head-mast | reserved / not Digicon head-mast | reserved / not Digicon head-mast | reserved / not Digicon head-mast</t>
         </is>
       </c>
     </row>
@@ -9168,7 +9168,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Princess North McKees Rocks Middle</t>
+          <t>Princess North McKees Rocks Bottom</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
@@ -9208,7 +9208,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Princess North McKees Rocks Bottom</t>
+          <t>Princess East McKeesport</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
@@ -9448,7 +9448,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Princess South McKeesport Middle</t>
+          <t>Princess South McKeesport Bottom</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Princess South McKeesport Bottom</t>
+          <t>Princess East McKees Rocks</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
@@ -9504,6 +9504,86 @@
       <c r="H259" t="inlineStr">
         <is>
           <t>HART Digicon; MQTT track/signalhead/IH141; packed 141 (node 1 sig 9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>D1-OU3-3</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Princess / Helix DCC node</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>3</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Princess East K-1</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Searchlight Signal Head</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>5V</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>HART Digicon; MQTT track/signalhead/IH142; packed 142 (node 1 sig 10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>D1-OU3-4</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Princess / Helix DCC node</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>4</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Princess East K-2</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Searchlight Signal Head</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>5V</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>HART Digicon; MQTT track/signalhead/IH143; packed 143 (node 1 sig 11)</t>
         </is>
       </c>
     </row>
@@ -9520,7 +9600,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G161"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="15.6640625" bestFit="1" customWidth="1" min="3" max="3"/>
   </cols>
@@ -13734,7 +13814,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I85"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="7.33203125" bestFit="1" customWidth="1" min="2" max="2"/>

</xml_diff>